<commit_message>
feat: plantilla RaySafe con valores nominales precargados
- Replantilla Excel replica estructura del informe de trabajo:
  cols A-F valores nominales (grupo, toma, kV, mA, t, mAs) precargados
  cols G-T zona 'Pegar DATOS RAY SAFE X2 aqui' (No/Sensor/Fecha/Hora + 5 pares valor-unidad)
  Paso2_Principales con 20 tomas en 8 grupos, hojas clinicas con 3 filas
- Parser detecta plantilla Sievert (col A = 'Grupo') y lee RaySafe
  desde offset 6 (col G) en lugar de col A del formato nativo

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantillas/plantilla-raysafe.xlsx
+++ b/public/plantillas/plantilla-raysafe.xlsx
@@ -400,284 +400,1068 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:T22"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="8.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="7.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="7.83203125" customWidth="1"/>
+    <col min="2" max="2" width="9.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="5.83203125" customWidth="1"/>
     <col min="8" max="8" width="7.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="5.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
-    <col min="13" max="13" width="13.83203125" customWidth="1"/>
-    <col min="14" max="14" width="11.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="9.83203125" customWidth="1"/>
+    <col min="12" max="12" width="7.83203125" customWidth="1"/>
+    <col min="13" max="13" width="9.83203125" customWidth="1"/>
+    <col min="14" max="14" width="7.83203125" customWidth="1"/>
+    <col min="15" max="15" width="9.83203125" customWidth="1"/>
+    <col min="16" max="16" width="7.83203125" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="12.83203125" customWidth="1"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1"/>
+    <col min="20" max="20" width="11.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Valores nominales</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+      <c r="G1" t="str">
+        <v>Pegar DATOS RAY SAFE X2 aqui</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Grupo</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Toma no.</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Tensión (KV)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Corriente (mA)</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Tiempo (s)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Exposición (mAs)</v>
+      </c>
+      <c r="G2" t="str">
         <v>No.</v>
       </c>
-      <c r="B1" t="str">
+      <c r="H2" t="str">
         <v>Sensor</v>
       </c>
-      <c r="C1" t="str">
+      <c r="I2" t="str">
         <v>Fecha</v>
       </c>
-      <c r="D1" t="str">
+      <c r="J2" t="str">
         <v>Hora</v>
       </c>
-      <c r="E1" t="str">
-        <v>kVp</v>
-      </c>
-      <c r="F1" t="str">
-        <v/>
-      </c>
-      <c r="G1" t="str">
-        <v>mGy</v>
-      </c>
-      <c r="H1" t="str">
-        <v/>
-      </c>
-      <c r="I1" t="str">
-        <v>s</v>
-      </c>
-      <c r="J1" t="str">
-        <v/>
-      </c>
-      <c r="K1" t="str">
-        <v>mm Al HVL</v>
-      </c>
-      <c r="L1" t="str">
-        <v/>
-      </c>
-      <c r="M1" t="str">
-        <v>mGy/min</v>
-      </c>
-      <c r="N1" t="str">
-        <v/>
+      <c r="K2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Unidad</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>60</v>
+      </c>
+      <c r="D3">
+        <v>100</v>
+      </c>
+      <c r="E3">
+        <v>0.1</v>
+      </c>
+      <c r="F3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>60</v>
+      </c>
+      <c r="D4">
+        <v>100</v>
+      </c>
+      <c r="E4">
+        <v>0.1</v>
+      </c>
+      <c r="F4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>60</v>
+      </c>
+      <c r="D5">
+        <v>100</v>
+      </c>
+      <c r="E5">
+        <v>0.1</v>
+      </c>
+      <c r="F5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>80</v>
+      </c>
+      <c r="D6">
+        <v>100</v>
+      </c>
+      <c r="E6">
+        <v>0.05</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>2</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7">
+        <v>80</v>
+      </c>
+      <c r="D7">
+        <v>100</v>
+      </c>
+      <c r="E7">
+        <v>0.05</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>2</v>
+      </c>
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8">
+        <v>80</v>
+      </c>
+      <c r="D8">
+        <v>100</v>
+      </c>
+      <c r="E8">
+        <v>0.05</v>
+      </c>
+      <c r="F8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9">
+        <v>80</v>
+      </c>
+      <c r="D9">
+        <v>200</v>
+      </c>
+      <c r="E9">
+        <v>0.05</v>
+      </c>
+      <c r="F9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>8</v>
+      </c>
+      <c r="C10">
+        <v>80</v>
+      </c>
+      <c r="D10">
+        <v>200</v>
+      </c>
+      <c r="E10">
+        <v>0.05</v>
+      </c>
+      <c r="F10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>3</v>
+      </c>
+      <c r="B11">
+        <v>9</v>
+      </c>
+      <c r="C11">
+        <v>80</v>
+      </c>
+      <c r="D11">
+        <v>200</v>
+      </c>
+      <c r="E11">
+        <v>0.05</v>
+      </c>
+      <c r="F11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>4</v>
+      </c>
+      <c r="B12">
+        <v>10</v>
+      </c>
+      <c r="C12">
+        <v>80</v>
+      </c>
+      <c r="D12">
+        <v>320</v>
+      </c>
+      <c r="E12">
+        <v>0.05</v>
+      </c>
+      <c r="F12">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>4</v>
+      </c>
+      <c r="B13">
+        <v>11</v>
+      </c>
+      <c r="C13">
+        <v>80</v>
+      </c>
+      <c r="D13">
+        <v>320</v>
+      </c>
+      <c r="E13">
+        <v>0.05</v>
+      </c>
+      <c r="F13">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>4</v>
+      </c>
+      <c r="B14">
+        <v>12</v>
+      </c>
+      <c r="C14">
+        <v>80</v>
+      </c>
+      <c r="D14">
+        <v>320</v>
+      </c>
+      <c r="E14">
+        <v>0.05</v>
+      </c>
+      <c r="F14">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>5</v>
+      </c>
+      <c r="B15">
+        <v>13</v>
+      </c>
+      <c r="C15">
+        <v>80</v>
+      </c>
+      <c r="D15">
+        <v>400</v>
+      </c>
+      <c r="E15">
+        <v>0.05</v>
+      </c>
+      <c r="F15">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>5</v>
+      </c>
+      <c r="B16">
+        <v>14</v>
+      </c>
+      <c r="C16">
+        <v>80</v>
+      </c>
+      <c r="D16">
+        <v>400</v>
+      </c>
+      <c r="E16">
+        <v>0.05</v>
+      </c>
+      <c r="F16">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>5</v>
+      </c>
+      <c r="B17">
+        <v>15</v>
+      </c>
+      <c r="C17">
+        <v>80</v>
+      </c>
+      <c r="D17">
+        <v>400</v>
+      </c>
+      <c r="E17">
+        <v>0.05</v>
+      </c>
+      <c r="F17">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>6</v>
+      </c>
+      <c r="B18">
+        <v>16</v>
+      </c>
+      <c r="C18">
+        <v>90</v>
+      </c>
+      <c r="D18">
+        <v>320</v>
+      </c>
+      <c r="E18">
+        <v>0.03125</v>
+      </c>
+      <c r="F18">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>6</v>
+      </c>
+      <c r="B19">
+        <v>17</v>
+      </c>
+      <c r="C19">
+        <v>90</v>
+      </c>
+      <c r="D19">
+        <v>320</v>
+      </c>
+      <c r="E19">
+        <v>0.03125</v>
+      </c>
+      <c r="F19">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>6</v>
+      </c>
+      <c r="B20">
+        <v>18</v>
+      </c>
+      <c r="C20">
+        <v>90</v>
+      </c>
+      <c r="D20">
+        <v>320</v>
+      </c>
+      <c r="E20">
+        <v>0.03125</v>
+      </c>
+      <c r="F20">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>7</v>
+      </c>
+      <c r="B21">
+        <v>19</v>
+      </c>
+      <c r="C21">
+        <v>80</v>
+      </c>
+      <c r="D21">
+        <v>140</v>
+      </c>
+      <c r="E21">
+        <v>0.0714286</v>
+      </c>
+      <c r="F21">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>8</v>
+      </c>
+      <c r="B22">
+        <v>20</v>
+      </c>
+      <c r="C22">
+        <v>80</v>
+      </c>
+      <c r="D22">
+        <v>50</v>
+      </c>
+      <c r="E22">
+        <v>5</v>
+      </c>
+      <c r="F22">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G1:T1"/>
+  </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T22"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:T5"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="8.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="7.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="7.83203125" customWidth="1"/>
+    <col min="2" max="2" width="9.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="5.83203125" customWidth="1"/>
     <col min="8" max="8" width="7.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="5.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
-    <col min="13" max="13" width="13.83203125" customWidth="1"/>
-    <col min="14" max="14" width="11.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="9.83203125" customWidth="1"/>
+    <col min="12" max="12" width="7.83203125" customWidth="1"/>
+    <col min="13" max="13" width="9.83203125" customWidth="1"/>
+    <col min="14" max="14" width="7.83203125" customWidth="1"/>
+    <col min="15" max="15" width="9.83203125" customWidth="1"/>
+    <col min="16" max="16" width="7.83203125" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="12.83203125" customWidth="1"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1"/>
+    <col min="20" max="20" width="11.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Valores nominales</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+      <c r="G1" t="str">
+        <v>Pegar DATOS RAY SAFE X2 aqui</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Grupo</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Toma no.</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Tensión (KV)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Corriente (mA)</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Tiempo (s)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Exposición (mAs)</v>
+      </c>
+      <c r="G2" t="str">
         <v>No.</v>
       </c>
-      <c r="B1" t="str">
+      <c r="H2" t="str">
         <v>Sensor</v>
       </c>
-      <c r="C1" t="str">
+      <c r="I2" t="str">
         <v>Fecha</v>
       </c>
-      <c r="D1" t="str">
+      <c r="J2" t="str">
         <v>Hora</v>
       </c>
-      <c r="E1" t="str">
-        <v>kVp</v>
-      </c>
-      <c r="F1" t="str">
-        <v/>
-      </c>
-      <c r="G1" t="str">
-        <v>mGy</v>
-      </c>
-      <c r="H1" t="str">
-        <v/>
-      </c>
-      <c r="I1" t="str">
-        <v>s</v>
-      </c>
-      <c r="J1" t="str">
-        <v/>
-      </c>
-      <c r="K1" t="str">
-        <v>mm Al HVL</v>
-      </c>
-      <c r="L1" t="str">
-        <v/>
-      </c>
-      <c r="M1" t="str">
-        <v>mGy/min</v>
-      </c>
-      <c r="N1" t="str">
+      <c r="K2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Unidad</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Extremidad</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Torax AP</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Columna AP</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G1:T1"/>
+  </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:T5"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="8.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="7.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="7.83203125" customWidth="1"/>
+    <col min="2" max="2" width="9.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="5.83203125" customWidth="1"/>
     <col min="8" max="8" width="7.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="5.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
-    <col min="13" max="13" width="13.83203125" customWidth="1"/>
-    <col min="14" max="14" width="11.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="9.83203125" customWidth="1"/>
+    <col min="12" max="12" width="7.83203125" customWidth="1"/>
+    <col min="13" max="13" width="9.83203125" customWidth="1"/>
+    <col min="14" max="14" width="7.83203125" customWidth="1"/>
+    <col min="15" max="15" width="9.83203125" customWidth="1"/>
+    <col min="16" max="16" width="7.83203125" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="12.83203125" customWidth="1"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1"/>
+    <col min="20" max="20" width="11.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Valores nominales</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+      <c r="G1" t="str">
+        <v>Pegar DATOS RAY SAFE X2 aqui</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Grupo</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Toma no.</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Tensión (KV)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Corriente (mA)</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Tiempo (s)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Exposición (mAs)</v>
+      </c>
+      <c r="G2" t="str">
         <v>No.</v>
       </c>
-      <c r="B1" t="str">
+      <c r="H2" t="str">
         <v>Sensor</v>
       </c>
-      <c r="C1" t="str">
+      <c r="I2" t="str">
         <v>Fecha</v>
       </c>
-      <c r="D1" t="str">
+      <c r="J2" t="str">
         <v>Hora</v>
       </c>
-      <c r="E1" t="str">
-        <v>kVp</v>
-      </c>
-      <c r="F1" t="str">
-        <v/>
-      </c>
-      <c r="G1" t="str">
-        <v>mGy</v>
-      </c>
-      <c r="H1" t="str">
-        <v/>
-      </c>
-      <c r="I1" t="str">
-        <v>s</v>
-      </c>
-      <c r="J1" t="str">
-        <v/>
-      </c>
-      <c r="K1" t="str">
-        <v>mm Al HVL</v>
-      </c>
-      <c r="L1" t="str">
-        <v/>
-      </c>
-      <c r="M1" t="str">
-        <v>mGy/min</v>
-      </c>
-      <c r="N1" t="str">
+      <c r="K2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Unidad</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Extremidad</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Torax AP</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Columna AP</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G1:T1"/>
+  </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:T5"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="8.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="7.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="7.83203125" customWidth="1"/>
+    <col min="2" max="2" width="9.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="5.83203125" customWidth="1"/>
     <col min="8" max="8" width="7.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="5.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
-    <col min="13" max="13" width="13.83203125" customWidth="1"/>
-    <col min="14" max="14" width="11.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="9.83203125" customWidth="1"/>
+    <col min="12" max="12" width="7.83203125" customWidth="1"/>
+    <col min="13" max="13" width="9.83203125" customWidth="1"/>
+    <col min="14" max="14" width="7.83203125" customWidth="1"/>
+    <col min="15" max="15" width="9.83203125" customWidth="1"/>
+    <col min="16" max="16" width="7.83203125" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="12.83203125" customWidth="1"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1"/>
+    <col min="20" max="20" width="11.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Valores nominales</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+      <c r="G1" t="str">
+        <v>Pegar DATOS RAY SAFE X2 aqui</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Grupo</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Toma no.</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Tensión (KV)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Corriente (mA)</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Tiempo (s)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Exposición (mAs)</v>
+      </c>
+      <c r="G2" t="str">
         <v>No.</v>
       </c>
-      <c r="B1" t="str">
+      <c r="H2" t="str">
         <v>Sensor</v>
       </c>
-      <c r="C1" t="str">
+      <c r="I2" t="str">
         <v>Fecha</v>
       </c>
-      <c r="D1" t="str">
+      <c r="J2" t="str">
         <v>Hora</v>
       </c>
-      <c r="E1" t="str">
-        <v>kVp</v>
-      </c>
-      <c r="F1" t="str">
-        <v/>
-      </c>
-      <c r="G1" t="str">
-        <v>mGy</v>
-      </c>
-      <c r="H1" t="str">
-        <v/>
-      </c>
-      <c r="I1" t="str">
-        <v>s</v>
-      </c>
-      <c r="J1" t="str">
-        <v/>
-      </c>
-      <c r="K1" t="str">
-        <v>mm Al HVL</v>
-      </c>
-      <c r="L1" t="str">
-        <v/>
-      </c>
-      <c r="M1" t="str">
-        <v>mGy/min</v>
-      </c>
-      <c r="N1" t="str">
+      <c r="K2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Unidad</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Unidad</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Extremidad</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Torax AP</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Columna AP</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G1:T1"/>
+  </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>